<commit_message>
the script with the database script V1 and fixes
</commit_message>
<xml_diff>
--- a/joined/saber11_dataframe_quality.xlsx
+++ b/joined/saber11_dataframe_quality.xlsx
@@ -877,19 +877,19 @@
         <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D10">
-        <v>5681596</v>
+        <v>6665246</v>
       </c>
       <c r="E10">
-        <v>85.23999999999999</v>
+        <v>100</v>
       </c>
       <c r="F10">
-        <v>983650</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>14.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -900,19 +900,19 @@
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D11">
-        <v>5681663</v>
+        <v>6665246</v>
       </c>
       <c r="E11">
-        <v>85.23999999999999</v>
+        <v>100</v>
       </c>
       <c r="F11">
-        <v>983583</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>14.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -923,19 +923,19 @@
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D12">
-        <v>5681663</v>
+        <v>6665246</v>
       </c>
       <c r="E12">
-        <v>85.23999999999999</v>
+        <v>100</v>
       </c>
       <c r="F12">
-        <v>983583</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>14.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -946,19 +946,19 @@
         <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D13">
-        <v>5681663</v>
+        <v>6665246</v>
       </c>
       <c r="E13">
-        <v>85.23999999999999</v>
+        <v>100</v>
       </c>
       <c r="F13">
-        <v>983583</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>14.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -969,19 +969,19 @@
         <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D14">
-        <v>5681662</v>
+        <v>6665246</v>
       </c>
       <c r="E14">
-        <v>85.23999999999999</v>
+        <v>100</v>
       </c>
       <c r="F14">
-        <v>983584</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>14.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1222,19 +1222,19 @@
         <v>29</v>
       </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D25">
-        <v>6663540</v>
+        <v>6665246</v>
       </c>
       <c r="E25">
-        <v>99.97</v>
+        <v>100</v>
       </c>
       <c r="F25">
-        <v>1706</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>0.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1245,19 +1245,19 @@
         <v>30</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D26">
-        <v>6663540</v>
+        <v>6665246</v>
       </c>
       <c r="E26">
-        <v>99.97</v>
+        <v>100</v>
       </c>
       <c r="F26">
-        <v>1706</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>0.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1268,19 +1268,19 @@
         <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D27">
-        <v>6651431</v>
+        <v>6665246</v>
       </c>
       <c r="E27">
-        <v>99.79000000000001</v>
+        <v>100</v>
       </c>
       <c r="F27">
-        <v>13815</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>0.21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1291,19 +1291,19 @@
         <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D28">
-        <v>6651431</v>
+        <v>6665246</v>
       </c>
       <c r="E28">
-        <v>99.79000000000001</v>
+        <v>100</v>
       </c>
       <c r="F28">
-        <v>13815</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>0.21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:7">

</xml_diff>